<commit_message>
Harmonize Sharpe ratio definition across Part II outputs
</commit_message>
<xml_diff>
--- a/outputs/excel/Part_II_results_filled.xlsx
+++ b/outputs/excel/Part_II_results_filled.xlsx
@@ -645,19 +645,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07171541381849046</v>
+        <v>0.07332339153529552</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1028178144011976</v>
+        <v>0.1046682011341537</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5275390663999439</v>
+        <v>0.5335755361240458</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.06823747759859851</v>
+        <v>-0.07227712498425057</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1342691177382868</v>
+        <v>0.1406317580718351</v>
       </c>
     </row>
     <row r="4">
@@ -689,19 +689,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1145626386679471</v>
+        <v>0.1125246016596191</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1762822292317981</v>
+        <v>0.1843343777484657</v>
       </c>
       <c r="D5" t="n">
-        <v>0.5507511397548986</v>
+        <v>0.5156368704557077</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.1683417910390196</v>
+        <v>-0.1822807470465652</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1450830455831827</v>
+        <v>0.1428412278334507</v>
       </c>
     </row>
     <row r="6">
@@ -711,19 +711,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1228324859604887</v>
+        <v>0.1152005249527049</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1784114085132021</v>
+        <v>0.1850587640012618</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5905311035795814</v>
+        <v>0.5280783403051293</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1685355403138382</v>
+        <v>-0.1861834873545179</v>
       </c>
       <c r="F6" t="n">
-        <v>0.143921863328095</v>
+        <v>0.1418298865892806</v>
       </c>
     </row>
   </sheetData>
@@ -800,16 +800,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>202.7640304512715</v>
+        <v>215.0528532162726</v>
       </c>
       <c r="C3" t="n">
-        <v>141.6676605599269</v>
+        <v>141.6676605599105</v>
       </c>
       <c r="D3" t="n">
-        <v>10.35626882742563</v>
+        <v>10.35626882742002</v>
       </c>
       <c r="E3" t="n">
-        <v>317.4166731412528</v>
+        <v>317.4166731403949</v>
       </c>
     </row>
     <row r="4">
@@ -838,16 +838,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>297.9517803714577</v>
+        <v>277.161042234068</v>
       </c>
       <c r="C5" t="n">
-        <v>259.126588967134</v>
+        <v>259.1257936012718</v>
       </c>
       <c r="D5" t="n">
-        <v>29.19194536654583</v>
+        <v>29.18240079847147</v>
       </c>
       <c r="E5" t="n">
-        <v>335.2830737583552</v>
+        <v>335.2830737584275</v>
       </c>
     </row>
     <row r="6">
@@ -857,16 +857,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>227.4889292626653</v>
+        <v>220.0334513823177</v>
       </c>
       <c r="C6" t="n">
-        <v>189.3007821765071</v>
+        <v>189.2685148658943</v>
       </c>
       <c r="D6" t="n">
-        <v>29.02707523862644</v>
+        <v>28.63986548206901</v>
       </c>
       <c r="E6" t="n">
-        <v>326.8168088754676</v>
+        <v>326.8168088848459</v>
       </c>
     </row>
   </sheetData>
@@ -926,16 +926,16 @@
         <v>194.7899575384342</v>
       </c>
       <c r="C2" t="n">
-        <v>111.7724840784875</v>
+        <v>110.9010195926205</v>
       </c>
       <c r="D2" t="n">
         <v>441.0575187854348</v>
       </c>
       <c r="E2" t="n">
-        <v>59.68978283113881</v>
+        <v>60.4702577428413</v>
       </c>
       <c r="F2" t="n">
-        <v>58.84868382880503</v>
+        <v>58.0523147301102</v>
       </c>
     </row>
     <row r="3">
@@ -946,16 +946,16 @@
         <v>266.6235239865563</v>
       </c>
       <c r="C3" t="n">
-        <v>136.6687615170862</v>
+        <v>140.7258137779986</v>
       </c>
       <c r="D3" t="n">
         <v>528.5450842326879</v>
       </c>
       <c r="E3" t="n">
-        <v>446.2476233036558</v>
+        <v>414.6939177246578</v>
       </c>
       <c r="F3" t="n">
-        <v>570.3129552489886</v>
+        <v>539.3006628746755</v>
       </c>
     </row>
     <row r="4">
@@ -966,16 +966,16 @@
         <v>48.15012288745206</v>
       </c>
       <c r="C4" t="n">
-        <v>15.25250187346307</v>
+        <v>14.69822714016272</v>
       </c>
       <c r="D4" t="n">
         <v>421.4507323352148</v>
       </c>
       <c r="E4" t="n">
-        <v>187.6604216610098</v>
+        <v>188.6382136595411</v>
       </c>
       <c r="F4" t="n">
-        <v>270.6595266225676</v>
+        <v>254.1437107099937</v>
       </c>
     </row>
     <row r="5">
@@ -986,16 +986,16 @@
         <v>149.5742439901542</v>
       </c>
       <c r="C5" t="n">
-        <v>30.71386217205391</v>
+        <v>31.55676347630432</v>
       </c>
       <c r="D5" t="n">
         <v>579.1998019012192</v>
       </c>
       <c r="E5" t="n">
-        <v>239.4220819667919</v>
+        <v>240.7757059792442</v>
       </c>
       <c r="F5" t="n">
-        <v>194.0870235941808</v>
+        <v>197.1200520883967</v>
       </c>
     </row>
     <row r="6">
@@ -1006,16 +1006,16 @@
         <v>276.9135276767599</v>
       </c>
       <c r="C6" t="n">
-        <v>58.33097907781649</v>
+        <v>50.6128047118702</v>
       </c>
       <c r="D6" t="n">
         <v>525.289561353253</v>
       </c>
       <c r="E6" t="n">
-        <v>387.007225201392</v>
+        <v>319.1201790272189</v>
       </c>
       <c r="F6" t="n">
-        <v>306.4309932275833</v>
+        <v>287.5081087607812</v>
       </c>
     </row>
     <row r="7">
@@ -1026,16 +1026,16 @@
         <v>1043.079454641516</v>
       </c>
       <c r="C7" t="n">
-        <v>579.8438143212527</v>
+        <v>640.8419121852789</v>
       </c>
       <c r="D7" t="n">
         <v>431.0774260152605</v>
       </c>
       <c r="E7" t="n">
-        <v>320.1639253043247</v>
+        <v>250.6752429790911</v>
       </c>
       <c r="F7" t="n">
-        <v>253.327353858385</v>
+        <v>231.03179800776</v>
       </c>
     </row>
     <row r="8">
@@ -1046,16 +1046,16 @@
         <v>557.4728077117604</v>
       </c>
       <c r="C8" t="n">
-        <v>224.5030701513384</v>
+        <v>224.0437304280637</v>
       </c>
       <c r="D8" t="n">
         <v>512.2414196937137</v>
       </c>
       <c r="E8" t="n">
-        <v>308.9134800270414</v>
+        <v>289.9670071083669</v>
       </c>
       <c r="F8" t="n">
-        <v>189.6718828487807</v>
+        <v>170.1346895971309</v>
       </c>
     </row>
     <row r="9">
@@ -1066,16 +1066,16 @@
         <v>334.7395376486194</v>
       </c>
       <c r="C9" t="n">
-        <v>158.580251090365</v>
+        <v>204.2587378164906</v>
       </c>
       <c r="D9" t="n">
         <v>307.5391351231141</v>
       </c>
       <c r="E9" t="n">
-        <v>263.7239601185275</v>
+        <v>175.4977370051547</v>
       </c>
       <c r="F9" t="n">
-        <v>182.1705532890983</v>
+        <v>145.9746040796286</v>
       </c>
     </row>
     <row r="10">
@@ -1086,16 +1086,16 @@
         <v>543.3272306662957</v>
       </c>
       <c r="C10" t="n">
-        <v>385.5437107842531</v>
+        <v>418.5838427926512</v>
       </c>
       <c r="D10" t="n">
         <v>433.3362454779038</v>
       </c>
       <c r="E10" t="n">
-        <v>229.4178979364869</v>
+        <v>229.3882824945441</v>
       </c>
       <c r="F10" t="n">
-        <v>152.2558396671826</v>
+        <v>152.7770702527456</v>
       </c>
     </row>
     <row r="11">
@@ -1106,16 +1106,16 @@
         <v>465.0597788716375</v>
       </c>
       <c r="C11" t="n">
-        <v>235.2137807372506</v>
+        <v>258.0693320965144</v>
       </c>
       <c r="D11" t="n">
         <v>342.0015494139942</v>
       </c>
       <c r="E11" t="n">
-        <v>239.2666459570603</v>
+        <v>234.4245028969621</v>
       </c>
       <c r="F11" t="n">
-        <v>152.5770825791411</v>
+        <v>146.9387240074248</v>
       </c>
     </row>
     <row r="12">
@@ -1126,16 +1126,16 @@
         <v>593.2080920590038</v>
       </c>
       <c r="C12" t="n">
-        <v>263.0487886734705</v>
+        <v>270.1163453679125</v>
       </c>
       <c r="D12" t="n">
         <v>322.7076762699301</v>
       </c>
       <c r="E12" t="n">
-        <v>625.9445073930414</v>
+        <v>627.0832077330103</v>
       </c>
       <c r="F12" t="n">
-        <v>296.7243663732478</v>
+        <v>296.8296311341641</v>
       </c>
     </row>
     <row r="13">
@@ -1146,16 +1146,16 @@
         <v>436.4530804900155</v>
       </c>
       <c r="C13" t="n">
-        <v>233.6963609384211</v>
+        <v>216.2257092094042</v>
       </c>
       <c r="D13" t="n">
         <v>306.3234167573739</v>
       </c>
       <c r="E13" t="n">
-        <v>267.9638127570215</v>
+        <v>295.1982524581828</v>
       </c>
       <c r="F13" t="n">
-        <v>102.8008900140232</v>
+        <v>160.5900503450013</v>
       </c>
     </row>
   </sheetData>
@@ -1215,16 +1215,16 @@
         <v>112.5405350883483</v>
       </c>
       <c r="C2" t="n">
-        <v>56.27026754421033</v>
+        <v>56.2702675441743</v>
       </c>
       <c r="D2" t="n">
         <v>403.4775418213042</v>
       </c>
       <c r="E2" t="n">
-        <v>29.19194536654583</v>
+        <v>29.18240079847147</v>
       </c>
       <c r="F2" t="n">
-        <v>29.02707523862644</v>
+        <v>28.63986548206901</v>
       </c>
     </row>
     <row r="3">
@@ -1235,16 +1235,16 @@
         <v>116.5270570478041</v>
       </c>
       <c r="C3" t="n">
-        <v>58.26352852398119</v>
+        <v>58.26352852390227</v>
       </c>
       <c r="D3" t="n">
         <v>515.9160610451851</v>
       </c>
       <c r="E3" t="n">
-        <v>257.9580305140915</v>
+        <v>257.9580305245165</v>
       </c>
       <c r="F3" t="n">
-        <v>326.8168088754676</v>
+        <v>326.8168088848459</v>
       </c>
     </row>
     <row r="4">
@@ -1255,16 +1255,16 @@
         <v>20.7125376548386</v>
       </c>
       <c r="C4" t="n">
-        <v>10.35626882742563</v>
+        <v>10.35626882742002</v>
       </c>
       <c r="D4" t="n">
         <v>425.6228843827011</v>
       </c>
       <c r="E4" t="n">
-        <v>212.8114421916814</v>
+        <v>212.8114421913568</v>
       </c>
       <c r="F4" t="n">
-        <v>294.1351261674326</v>
+        <v>294.1351279879058</v>
       </c>
     </row>
     <row r="5">
@@ -1275,16 +1275,16 @@
         <v>40.71024720836911</v>
       </c>
       <c r="C5" t="n">
-        <v>20.35512360418613</v>
+        <v>20.35512360418593</v>
       </c>
       <c r="D5" t="n">
         <v>665.0028746034002</v>
       </c>
       <c r="E5" t="n">
-        <v>332.5014373021155</v>
+        <v>332.5014373018474</v>
       </c>
       <c r="F5" t="n">
-        <v>264.7216151889005</v>
+        <v>264.7216151889717</v>
       </c>
     </row>
     <row r="6">
@@ -1295,16 +1295,16 @@
         <v>57.07206046352246</v>
       </c>
       <c r="C6" t="n">
-        <v>28.53603023166318</v>
+        <v>28.53603023176075</v>
       </c>
       <c r="D6" t="n">
         <v>613.1245771995201</v>
       </c>
       <c r="E6" t="n">
-        <v>306.5622885999029</v>
+        <v>306.5622885997811</v>
       </c>
       <c r="F6" t="n">
-        <v>238.2494536701087</v>
+        <v>238.2494536700623</v>
       </c>
     </row>
     <row r="7">
@@ -1315,16 +1315,16 @@
         <v>400.7348455851865</v>
       </c>
       <c r="C7" t="n">
-        <v>200.3674227925227</v>
+        <v>200.3674227926068</v>
       </c>
       <c r="D7" t="n">
         <v>542.7340818157821</v>
       </c>
       <c r="E7" t="n">
-        <v>271.3670409076273</v>
+        <v>271.3670409576399</v>
       </c>
       <c r="F7" t="n">
-        <v>214.4245083030771</v>
+        <v>214.4245083128846</v>
       </c>
     </row>
     <row r="8">
@@ -1335,16 +1335,16 @@
         <v>211.219022633161</v>
       </c>
       <c r="C8" t="n">
-        <v>105.6095113165007</v>
+        <v>105.609511316581</v>
       </c>
       <c r="D8" t="n">
         <v>670.566147516855</v>
       </c>
       <c r="E8" t="n">
-        <v>335.2830737583552</v>
+        <v>335.2830737584275</v>
       </c>
       <c r="F8" t="n">
-        <v>192.9820574727829</v>
+        <v>192.9820574727503</v>
       </c>
     </row>
     <row r="9">
@@ -1355,16 +1355,16 @@
         <v>253.8871418467655</v>
       </c>
       <c r="C9" t="n">
-        <v>126.9435709235813</v>
+        <v>126.9435709233901</v>
       </c>
       <c r="D9" t="n">
         <v>603.5017893543784</v>
       </c>
       <c r="E9" t="n">
-        <v>301.7508946771541</v>
+        <v>301.7508947065706</v>
       </c>
       <c r="F9" t="n">
-        <v>173.6838517254001</v>
+        <v>173.6838517260836</v>
       </c>
     </row>
     <row r="10">
@@ -1375,16 +1375,16 @@
         <v>365.5442860445737</v>
       </c>
       <c r="C10" t="n">
-        <v>182.7721430222206</v>
+        <v>182.7721430222859</v>
       </c>
       <c r="D10" t="n">
         <v>528.9304667311615</v>
       </c>
       <c r="E10" t="n">
-        <v>264.4652333620771</v>
+        <v>264.4652334020008</v>
       </c>
       <c r="F10" t="n">
-        <v>156.3154665530216</v>
+        <v>156.3154666363087</v>
       </c>
     </row>
     <row r="11">
@@ -1395,16 +1395,16 @@
         <v>594.1737755232857</v>
       </c>
       <c r="C11" t="n">
-        <v>297.0868877610731</v>
+        <v>297.0868877616484</v>
       </c>
       <c r="D11" t="n">
         <v>507.5056957196227</v>
       </c>
       <c r="E11" t="n">
-        <v>253.7528478598031</v>
+        <v>253.7528478780514</v>
       </c>
       <c r="F11" t="n">
-        <v>140.6839198976489</v>
+        <v>140.6839199046197</v>
       </c>
     </row>
     <row r="12">
@@ -1415,16 +1415,16 @@
         <v>634.8333462807853</v>
       </c>
       <c r="C12" t="n">
-        <v>317.4166731412528</v>
+        <v>317.4166731403949</v>
       </c>
       <c r="D12" t="n">
         <v>574.5692017896073</v>
       </c>
       <c r="E12" t="n">
-        <v>287.2846008947688</v>
+        <v>287.2846008948187</v>
       </c>
       <c r="F12" t="n">
-        <v>126.6155279078397</v>
+        <v>126.6155279078713</v>
       </c>
     </row>
     <row r="13">
@@ -1435,16 +1435,16 @@
         <v>592.0689980611453</v>
       </c>
       <c r="C13" t="n">
-        <v>296.0344990305058</v>
+        <v>296.0344990305749</v>
       </c>
       <c r="D13" t="n">
         <v>513.1804643431068</v>
       </c>
       <c r="E13" t="n">
-        <v>256.5902321714855</v>
+        <v>256.5902322017791</v>
       </c>
       <c r="F13" t="n">
-        <v>113.9539751177789</v>
+        <v>113.9539752163584</v>
       </c>
     </row>
   </sheetData>
@@ -1504,16 +1504,16 @@
         <v>-0.03649865416421228</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.03583694804822943</v>
+        <v>-0.03736165726718697</v>
       </c>
       <c r="D2" t="n">
         <v>-0.07026498004277006</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.07311825813802261</v>
+        <v>-0.07325655637725262</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.07320855297460958</v>
+        <v>-0.07360057471981932</v>
       </c>
     </row>
     <row r="3">
@@ -1524,16 +1524,16 @@
         <v>0.01965962026518523</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01219822326774553</v>
+        <v>0.01377781392166122</v>
       </c>
       <c r="D3" t="n">
         <v>0.02077622686678488</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02438173433570073</v>
+        <v>0.02288857027022771</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02434401378639235</v>
+        <v>0.02324985107269244</v>
       </c>
     </row>
     <row r="4">
@@ -1544,16 +1544,16 @@
         <v>0.0155391281256913</v>
       </c>
       <c r="C4" t="n">
-        <v>0.01345191667802142</v>
+        <v>0.01417503753560567</v>
       </c>
       <c r="D4" t="n">
         <v>0.04467723574102896</v>
       </c>
       <c r="E4" t="n">
-        <v>0.03190233074373888</v>
+        <v>0.03179704154469569</v>
       </c>
       <c r="F4" t="n">
-        <v>0.03180206516786169</v>
+        <v>0.03144586117414425</v>
       </c>
     </row>
     <row r="5">
@@ -1564,16 +1564,16 @@
         <v>0.02734641306038766</v>
       </c>
       <c r="C5" t="n">
-        <v>0.02939733981400667</v>
+        <v>0.03052418383439543</v>
       </c>
       <c r="D5" t="n">
         <v>0.006795170125112241</v>
       </c>
       <c r="E5" t="n">
-        <v>0.04619244543120093</v>
+        <v>0.04513516461309551</v>
       </c>
       <c r="F5" t="n">
-        <v>0.04629958151883243</v>
+        <v>0.04508588967085344</v>
       </c>
     </row>
     <row r="6">
@@ -1584,16 +1584,16 @@
         <v>0.006262336674770144</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01423900943620347</v>
+        <v>0.01363754937134583</v>
       </c>
       <c r="D6" t="n">
         <v>0.04339620179990861</v>
       </c>
       <c r="E6" t="n">
-        <v>0.05926982102994279</v>
+        <v>0.06018479457176484</v>
       </c>
       <c r="F6" t="n">
-        <v>0.05936640262864885</v>
+        <v>0.06015972171982917</v>
       </c>
     </row>
     <row r="7">
@@ -1604,16 +1604,16 @@
         <v>0.01320043855385788</v>
       </c>
       <c r="C7" t="n">
-        <v>0.01281598215681805</v>
+        <v>0.01287251278935389</v>
       </c>
       <c r="D7" t="n">
         <v>0.03569530268075231</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01159517919140444</v>
+        <v>0.01112997232338329</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01154569423576836</v>
+        <v>0.01114131533930648</v>
       </c>
     </row>
     <row r="8">
@@ -1624,16 +1624,16 @@
         <v>0.00634089399497464</v>
       </c>
       <c r="C8" t="n">
-        <v>0.01164236179070497</v>
+        <v>0.01189168483251219</v>
       </c>
       <c r="D8" t="n">
         <v>-0.007361026260429289</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.02245558321344751</v>
+        <v>-0.02317912608453078</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.02246866039835796</v>
+        <v>-0.02308311579065594</v>
       </c>
     </row>
     <row r="9">
@@ -1644,16 +1644,16 @@
         <v>0.03877121196595493</v>
       </c>
       <c r="C9" t="n">
-        <v>0.03454856280021416</v>
+        <v>0.03552613815674961</v>
       </c>
       <c r="D9" t="n">
         <v>0.02463494349528241</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01747356683840885</v>
+        <v>0.01605343255200611</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01739307923278254</v>
+        <v>0.01644710268900956</v>
       </c>
     </row>
     <row r="10">
@@ -1664,16 +1664,16 @@
         <v>-0.03050354350157332</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.02923387887097797</v>
+        <v>-0.03013574152666567</v>
       </c>
       <c r="D10" t="n">
         <v>-0.07531135274733532</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1560780519893695</v>
+        <v>-0.1575253214834718</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.1565683420859283</v>
+        <v>-0.1570734619752157</v>
       </c>
     </row>
     <row r="11">
@@ -1684,16 +1684,16 @@
         <v>0.02281906843041514</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0190038915701594</v>
+        <v>0.01959022112292449</v>
       </c>
       <c r="D11" t="n">
         <v>0.00775658866595595</v>
       </c>
       <c r="E11" t="n">
-        <v>0.03536778451554821</v>
+        <v>0.03517549141194114</v>
       </c>
       <c r="F11" t="n">
-        <v>0.03538548909120634</v>
+        <v>0.03563551888871314</v>
       </c>
     </row>
     <row r="12">
@@ -1704,16 +1704,16 @@
         <v>-0.01887228565706454</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.018357075905775</v>
+        <v>-0.01807993353111678</v>
       </c>
       <c r="D12" t="n">
         <v>-0.02126323916811964</v>
       </c>
       <c r="E12" t="n">
-        <v>0.006076084215550987</v>
+        <v>0.005339168604568484</v>
       </c>
       <c r="F12" t="n">
-        <v>0.006101444960933289</v>
+        <v>0.00534842877553827</v>
       </c>
     </row>
     <row r="13">
@@ -1724,16 +1724,16 @@
         <v>-0.03116883433505653</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.03172168307072112</v>
+        <v>-0.03075619716078289</v>
       </c>
       <c r="D13" t="n">
         <v>-0.06901007205913473</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.05139344135891089</v>
+        <v>-0.05175106580416117</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.05135818990087557</v>
+        <v>-0.05081637896891565</v>
       </c>
     </row>
     <row r="14">
@@ -1744,16 +1744,16 @@
         <v>0.01371152603973757</v>
       </c>
       <c r="C14" t="n">
-        <v>0.01469822385649029</v>
+        <v>0.01224869195025476</v>
       </c>
       <c r="D14" t="n">
         <v>0.007339331453900047</v>
       </c>
       <c r="E14" t="n">
-        <v>0.06813675257779726</v>
+        <v>0.0657874101487719</v>
       </c>
       <c r="F14" t="n">
-        <v>0.06709635179757233</v>
+        <v>0.06565676131731497</v>
       </c>
     </row>
     <row r="15">
@@ -1764,16 +1764,16 @@
         <v>0.03508508435636881</v>
       </c>
       <c r="C15" t="n">
-        <v>0.03383916362974454</v>
+        <v>0.03582433188680637</v>
       </c>
       <c r="D15" t="n">
         <v>0.04141390361404322</v>
       </c>
       <c r="E15" t="n">
-        <v>0.03478422341992417</v>
+        <v>0.03789171497276372</v>
       </c>
       <c r="F15" t="n">
-        <v>0.03525971482420634</v>
+        <v>0.03803780695783255</v>
       </c>
     </row>
     <row r="16">
@@ -1784,16 +1784,16 @@
         <v>-0.0007744917573539734</v>
       </c>
       <c r="C16" t="n">
-        <v>0.002593154574665255</v>
+        <v>0.002831938410308403</v>
       </c>
       <c r="D16" t="n">
         <v>-0.03181535717049088</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.03813180572012914</v>
+        <v>-0.0364958315298366</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.04064745810295668</v>
+        <v>-0.03771035895374326</v>
       </c>
     </row>
     <row r="17">
@@ -1804,16 +1804,16 @@
         <v>0.0270682666372253</v>
       </c>
       <c r="C17" t="n">
-        <v>0.02869143393826873</v>
+        <v>0.02855852530245956</v>
       </c>
       <c r="D17" t="n">
         <v>0.05520842262682887</v>
       </c>
       <c r="E17" t="n">
-        <v>0.06733972136056479</v>
+        <v>0.06644182183208111</v>
       </c>
       <c r="F17" t="n">
-        <v>0.06882376658597833</v>
+        <v>0.06681425582011186</v>
       </c>
     </row>
     <row r="18">
@@ -1824,16 +1824,16 @@
         <v>-0.04631065920667646</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.03849598310702151</v>
+        <v>-0.03967235859597721</v>
       </c>
       <c r="D18" t="n">
         <v>-0.04519396145635353</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.03773470510612172</v>
+        <v>-0.03919595203485973</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.03806006397342146</v>
+        <v>-0.03861544052145331</v>
       </c>
     </row>
     <row r="19">
@@ -1844,16 +1844,16 @@
         <v>-0.0277041300910287</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.02244104422194854</v>
+        <v>-0.02199331813374594</v>
       </c>
       <c r="D19" t="n">
         <v>-0.01671837114782021</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.002887142868189026</v>
+        <v>-0.003850193700995937</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.003062698570913687</v>
+        <v>-0.003977441097325965</v>
       </c>
     </row>
     <row r="20">
@@ -1864,16 +1864,16 @@
         <v>0.01860379034121998</v>
       </c>
       <c r="C20" t="n">
-        <v>0.01819043713561493</v>
+        <v>0.0202998524612642</v>
       </c>
       <c r="D20" t="n">
         <v>-0.05212452092794789</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.06218172452000967</v>
+        <v>-0.06076817884750284</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.06254375915131373</v>
+        <v>-0.06025435276601365</v>
       </c>
     </row>
     <row r="21">
@@ -1884,16 +1884,16 @@
         <v>-0.07187086903754682</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.06823747759859851</v>
+        <v>-0.07227712498425057</v>
       </c>
       <c r="D21" t="n">
         <v>-0.08464422338745563</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.05556234651244535</v>
+        <v>-0.05758545655971122</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.05779645467437405</v>
+        <v>-0.05979561209896612</v>
       </c>
     </row>
     <row r="22">
@@ -1904,16 +1904,16 @@
         <v>-0.01833165785473283</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.0169662751124159</v>
+        <v>-0.01759246900095462</v>
       </c>
       <c r="D22" t="n">
         <v>-0.02493133275277176</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.02871975194683649</v>
+        <v>-0.03049601451085903</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.02909487078301824</v>
+        <v>-0.03024732631044863</v>
       </c>
     </row>
     <row r="23">
@@ -1924,16 +1924,16 @@
         <v>0.03511363660085631</v>
       </c>
       <c r="C23" t="n">
-        <v>0.03406816775133001</v>
+        <v>0.03556934858961231</v>
       </c>
       <c r="D23" t="n">
         <v>0.06491029329859194</v>
       </c>
       <c r="E23" t="n">
-        <v>0.04434601578507215</v>
+        <v>0.04162230153904632</v>
       </c>
       <c r="F23" t="n">
-        <v>0.04607475410277662</v>
+        <v>0.04300440470331652</v>
       </c>
     </row>
     <row r="24">
@@ -1944,16 +1944,16 @@
         <v>-0.02591029444208056</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.02504651871942114</v>
+        <v>-0.02737033777081602</v>
       </c>
       <c r="D24" t="n">
         <v>-0.0357558144902735</v>
       </c>
       <c r="E24" t="n">
-        <v>-0.0264160043128073</v>
+        <v>-0.02926510997772758</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.02730593628786134</v>
+        <v>-0.02896719754202937</v>
       </c>
     </row>
     <row r="25">
@@ -1964,16 +1964,16 @@
         <v>-0.01596111878380158</v>
       </c>
       <c r="C25" t="n">
-        <v>-0.01694537394729582</v>
+        <v>-0.01907035781319561</v>
       </c>
       <c r="D25" t="n">
         <v>-0.02106535603086771</v>
       </c>
       <c r="E25" t="n">
-        <v>0.006407367722122904</v>
+        <v>0.00710173220557718</v>
       </c>
       <c r="F25" t="n">
-        <v>0.006578769332808185</v>
+        <v>0.00882000419104513</v>
       </c>
     </row>
     <row r="26">
@@ -1984,16 +1984,16 @@
         <v>0.04473406834969725</v>
       </c>
       <c r="C26" t="n">
-        <v>0.03911248833830576</v>
+        <v>0.0421544999269632</v>
       </c>
       <c r="D26" t="n">
         <v>-0.04230023559388479</v>
       </c>
       <c r="E26" t="n">
-        <v>0.002424970589725142</v>
+        <v>-0.002392967628802228</v>
       </c>
       <c r="F26" t="n">
-        <v>0.002948856428149755</v>
+        <v>0.0008256656599966716</v>
       </c>
     </row>
     <row r="27">
@@ -2004,16 +2004,16 @@
         <v>-0.0024388990608279</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.006098731554785044</v>
+        <v>-0.002039081985481084</v>
       </c>
       <c r="D27" t="n">
         <v>-0.0078763026838919</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0081034271141666</v>
+        <v>0.006315118570159105</v>
       </c>
       <c r="F27" t="n">
-        <v>0.009102225058918424</v>
+        <v>0.007893923637439564</v>
       </c>
     </row>
     <row r="28">
@@ -2024,16 +2024,16 @@
         <v>0.08147079497264535</v>
       </c>
       <c r="C28" t="n">
-        <v>0.0801506402192091</v>
+        <v>0.07981986866070806</v>
       </c>
       <c r="D28" t="n">
         <v>0.1344288672572242</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1166502035718451</v>
+        <v>0.1182532077726947</v>
       </c>
       <c r="F28" t="n">
-        <v>0.118993980433926</v>
+        <v>0.1181081714684147</v>
       </c>
     </row>
     <row r="29">
@@ -2044,16 +2044,16 @@
         <v>-0.02014093371819024</v>
       </c>
       <c r="C29" t="n">
-        <v>-0.01165548357395392</v>
+        <v>-0.01246586936707672</v>
       </c>
       <c r="D29" t="n">
         <v>0.019650899382275</v>
       </c>
       <c r="E29" t="n">
-        <v>0.02645106477308213</v>
+        <v>0.02909541353562789</v>
       </c>
       <c r="F29" t="n">
-        <v>0.03151124868180086</v>
+        <v>0.03274991477676818</v>
       </c>
     </row>
     <row r="30">
@@ -2064,16 +2064,16 @@
         <v>0.009053828166525842</v>
       </c>
       <c r="C30" t="n">
-        <v>0.005498211942158647</v>
+        <v>0.006373846988968433</v>
       </c>
       <c r="D30" t="n">
         <v>-0.03779392015602362</v>
       </c>
       <c r="E30" t="n">
-        <v>-0.03778625847608627</v>
+        <v>-0.03205071140640837</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.03471867844254368</v>
+        <v>-0.02863530604203775</v>
       </c>
     </row>
     <row r="31">
@@ -2084,16 +2084,16 @@
         <v>0.05887672707655323</v>
       </c>
       <c r="C31" t="n">
-        <v>0.06593504363087524</v>
+        <v>0.06626204320603615</v>
       </c>
       <c r="D31" t="n">
         <v>0.04977529648158455</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0363651689114482</v>
+        <v>0.04039866397915786</v>
       </c>
       <c r="F31" t="n">
-        <v>0.03612607183400744</v>
+        <v>0.03926001886541807</v>
       </c>
     </row>
     <row r="32">
@@ -2104,16 +2104,16 @@
         <v>0.01973485816907689</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0234884411895319</v>
+        <v>0.02476523749925926</v>
       </c>
       <c r="D32" t="n">
         <v>0.04574271959133058</v>
       </c>
       <c r="E32" t="n">
-        <v>0.03867915707787206</v>
+        <v>0.04176745049906821</v>
       </c>
       <c r="F32" t="n">
-        <v>0.03933296991326719</v>
+        <v>0.04111947693954078</v>
       </c>
     </row>
     <row r="33">
@@ -2124,16 +2124,16 @@
         <v>-0.01247481344690763</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.01096897563644837</v>
+        <v>-0.01320727610499802</v>
       </c>
       <c r="D33" t="n">
         <v>0.02043609851042295</v>
       </c>
       <c r="E33" t="n">
-        <v>0.01540882731603358</v>
+        <v>0.0202355030342207</v>
       </c>
       <c r="F33" t="n">
-        <v>0.01865771766580582</v>
+        <v>0.01926867728040566</v>
       </c>
     </row>
     <row r="34">
@@ -2144,16 +2144,16 @@
         <v>-0.005238919074118562</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.009456586091274399</v>
+        <v>-0.008361801458375364</v>
       </c>
       <c r="D34" t="n">
         <v>0.007018885117639503</v>
       </c>
       <c r="E34" t="n">
-        <v>-0.004872204035524092</v>
+        <v>-0.00342943633674741</v>
       </c>
       <c r="F34" t="n">
-        <v>-0.007225147498531996</v>
+        <v>-0.008661287620075897</v>
       </c>
     </row>
     <row r="35">
@@ -2164,16 +2164,16 @@
         <v>-0.0400479406719685</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.03652923610419312</v>
+        <v>-0.03593376317001352</v>
       </c>
       <c r="D35" t="n">
         <v>0.008182529362591296</v>
       </c>
       <c r="E35" t="n">
-        <v>-0.008477706854795796</v>
+        <v>-0.007951544215927643</v>
       </c>
       <c r="F35" t="n">
-        <v>-0.00848975653461998</v>
+        <v>-0.007932606748921938</v>
       </c>
     </row>
     <row r="36">
@@ -2184,16 +2184,16 @@
         <v>-0.07469915291397239</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.06065223526586361</v>
+        <v>-0.06241323134541987</v>
       </c>
       <c r="D36" t="n">
         <v>-0.03732341822162155</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.03108671725648269</v>
+        <v>-0.02435059425236712</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.02935317823300838</v>
+        <v>-0.02722865128738645</v>
       </c>
     </row>
     <row r="37">
@@ -2204,16 +2204,16 @@
         <v>-0.02434305449003699</v>
       </c>
       <c r="C37" t="n">
-        <v>-0.02839164876832674</v>
+        <v>-0.02736707284467131</v>
       </c>
       <c r="D37" t="n">
         <v>0.02032329511426291</v>
       </c>
       <c r="E37" t="n">
-        <v>-0.01860407281090657</v>
+        <v>-0.01661503160573919</v>
       </c>
       <c r="F37" t="n">
-        <v>-0.02469478222303541</v>
+        <v>-0.02403069928713195</v>
       </c>
     </row>
     <row r="38">
@@ -2224,16 +2224,16 @@
         <v>0.01357608550579243</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0134556192409739</v>
+        <v>0.01417672377316495</v>
       </c>
       <c r="D38" t="n">
         <v>0.04727385709321499</v>
       </c>
       <c r="E38" t="n">
-        <v>0.03912103245586114</v>
+        <v>0.03945763715162109</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0382536959593883</v>
+        <v>0.0422674653692132</v>
       </c>
     </row>
     <row r="39">
@@ -2244,16 +2244,16 @@
         <v>0.04708600796748979</v>
       </c>
       <c r="C39" t="n">
-        <v>0.04260321855354085</v>
+        <v>0.04173596850890277</v>
       </c>
       <c r="D39" t="n">
         <v>0.02665901511045048</v>
       </c>
       <c r="E39" t="n">
-        <v>0.05510393780759268</v>
+        <v>0.05558626374007132</v>
       </c>
       <c r="F39" t="n">
-        <v>0.05558609488906624</v>
+        <v>0.05406118167551828</v>
       </c>
     </row>
     <row r="40">
@@ -2264,16 +2264,16 @@
         <v>0.02018927446922038</v>
       </c>
       <c r="C40" t="n">
-        <v>0.02005744197466119</v>
+        <v>0.02007027196789638</v>
       </c>
       <c r="D40" t="n">
         <v>0.02028145574585162</v>
       </c>
       <c r="E40" t="n">
-        <v>0.04125322979768516</v>
+        <v>0.04074142679844683</v>
       </c>
       <c r="F40" t="n">
-        <v>0.04015246070620212</v>
+        <v>0.0398967251940629</v>
       </c>
     </row>
     <row r="41">
@@ -2284,16 +2284,16 @@
         <v>0.0003715564497607129</v>
       </c>
       <c r="C41" t="n">
-        <v>0.001118880602773986</v>
+        <v>0.001454174223234369</v>
       </c>
       <c r="D41" t="n">
         <v>0.01158976941153002</v>
       </c>
       <c r="E41" t="n">
-        <v>0.01673195583499676</v>
+        <v>0.01518967235351343</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0180916082389156</v>
+        <v>0.01691490842946677</v>
       </c>
     </row>
     <row r="42">
@@ -2304,16 +2304,16 @@
         <v>0.0554323768789813</v>
       </c>
       <c r="C42" t="n">
-        <v>0.0596976933178737</v>
+        <v>0.05670743840276841</v>
       </c>
       <c r="D42" t="n">
         <v>0.01504055287089303</v>
       </c>
       <c r="E42" t="n">
-        <v>-0.004861513695579758</v>
+        <v>-0.004396376810317501</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.001033674758481273</v>
+        <v>-0.001350980691600896</v>
       </c>
     </row>
     <row r="43">
@@ -2324,16 +2324,16 @@
         <v>0.0009013197658726451</v>
       </c>
       <c r="C43" t="n">
-        <v>0.0003421349700314879</v>
+        <v>-0.0001825776583792237</v>
       </c>
       <c r="D43" t="n">
         <v>0.001160368965973042</v>
       </c>
       <c r="E43" t="n">
-        <v>-0.00593091898387101</v>
+        <v>-0.005288124661346479</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.007368066133115681</v>
+        <v>-0.004169115062604829</v>
       </c>
     </row>
     <row r="44">
@@ -2344,16 +2344,16 @@
         <v>0.01066299611965773</v>
       </c>
       <c r="C44" t="n">
-        <v>0.008018888856579804</v>
+        <v>0.008055378990144071</v>
       </c>
       <c r="D44" t="n">
         <v>0.04799108027004863</v>
       </c>
       <c r="E44" t="n">
-        <v>0.05001798547176575</v>
+        <v>0.05191860248592045</v>
       </c>
       <c r="F44" t="n">
-        <v>0.05223393858966315</v>
+        <v>0.05383831511466171</v>
       </c>
     </row>
     <row r="45">
@@ -2364,16 +2364,16 @@
         <v>-0.004607831124146113</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.002461851798874589</v>
+        <v>-0.0005806595196995203</v>
       </c>
       <c r="D45" t="n">
         <v>0.02768204362181925</v>
       </c>
       <c r="E45" t="n">
-        <v>0.02421013350205706</v>
+        <v>0.02376859819383336</v>
       </c>
       <c r="F45" t="n">
-        <v>0.02313577364739735</v>
+        <v>0.02490420907785294</v>
       </c>
     </row>
     <row r="46">
@@ -2384,16 +2384,16 @@
         <v>0.007875082940049287</v>
       </c>
       <c r="C46" t="n">
-        <v>0.00707754196145445</v>
+        <v>0.0059999392727747</v>
       </c>
       <c r="D46" t="n">
         <v>-0.00570725226602121</v>
       </c>
       <c r="E46" t="n">
-        <v>-0.0008273518642137791</v>
+        <v>-0.002464791012258397</v>
       </c>
       <c r="F46" t="n">
-        <v>-0.005001473065013701</v>
+        <v>-0.006377432098985789</v>
       </c>
     </row>
     <row r="47">
@@ -2404,16 +2404,16 @@
         <v>0.007307510240592709</v>
       </c>
       <c r="C47" t="n">
-        <v>0.006805249407386832</v>
+        <v>0.004027579221483722</v>
       </c>
       <c r="D47" t="n">
         <v>0.03870562748930086</v>
       </c>
       <c r="E47" t="n">
-        <v>0.03983724572999789</v>
+        <v>0.04024742173200366</v>
       </c>
       <c r="F47" t="n">
-        <v>0.04079849836975017</v>
+        <v>0.04053694877347426</v>
       </c>
     </row>
     <row r="48">
@@ -2424,16 +2424,16 @@
         <v>0.01364089450924604</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02033861230255325</v>
+        <v>0.01739799609141037</v>
       </c>
       <c r="D48" t="n">
         <v>-0.005876212524494721</v>
       </c>
       <c r="E48" t="n">
-        <v>-0.001035061184141999</v>
+        <v>-0.003910078039012543</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.002414949333985752</v>
+        <v>-0.00813406929955918</v>
       </c>
     </row>
     <row r="49">
@@ -2444,16 +2444,16 @@
         <v>0.04628155692471259</v>
       </c>
       <c r="C49" t="n">
-        <v>0.04337079847063514</v>
+        <v>0.04326948151697872</v>
       </c>
       <c r="D49" t="n">
         <v>0.05104246015880655</v>
       </c>
       <c r="E49" t="n">
-        <v>0.04801442715318003</v>
+        <v>0.04708957091837177</v>
       </c>
       <c r="F49" t="n">
-        <v>0.04970340632443344</v>
+        <v>0.0476005296120016</v>
       </c>
     </row>
     <row r="50">
@@ -2464,16 +2464,16 @@
         <v>0.0372432126422939</v>
       </c>
       <c r="C50" t="n">
-        <v>0.03873964677614053</v>
+        <v>0.03530367229387137</v>
       </c>
       <c r="D50" t="n">
         <v>0.0893234684450967</v>
       </c>
       <c r="E50" t="n">
-        <v>0.08870410719862637</v>
+        <v>0.09803695603280757</v>
       </c>
       <c r="F50" t="n">
-        <v>0.08878775545142786</v>
+        <v>0.09932576490437603</v>
       </c>
     </row>
     <row r="51">
@@ -2484,16 +2484,16 @@
         <v>-0.02618760419048109</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.02087161829851764</v>
+        <v>-0.02508393017137738</v>
       </c>
       <c r="D51" t="n">
         <v>-0.04479130657071866</v>
       </c>
       <c r="E51" t="n">
-        <v>-0.04515455770569242</v>
+        <v>-0.0426573714924366</v>
       </c>
       <c r="F51" t="n">
-        <v>-0.04536763378353191</v>
+        <v>-0.04181569773488443</v>
       </c>
     </row>
     <row r="52">
@@ -2504,16 +2504,16 @@
         <v>0.01900678106808058</v>
       </c>
       <c r="C52" t="n">
-        <v>0.02197328360304294</v>
+        <v>0.01591378123372401</v>
       </c>
       <c r="D52" t="n">
         <v>-0.01880510215300218</v>
       </c>
       <c r="E52" t="n">
-        <v>-0.01826151409585659</v>
+        <v>-0.01078023015548961</v>
       </c>
       <c r="F52" t="n">
-        <v>-0.01826466315152269</v>
+        <v>-0.009977450827032932</v>
       </c>
     </row>
     <row r="53">
@@ -2524,16 +2524,16 @@
         <v>-0.002822531344317912</v>
       </c>
       <c r="C53" t="n">
-        <v>-0.01052513181417058</v>
+        <v>-0.008013841347053919</v>
       </c>
       <c r="D53" t="n">
         <v>-0.0006726306147162645</v>
       </c>
       <c r="E53" t="n">
-        <v>-0.00113258048850939</v>
+        <v>0.009623451842348186</v>
       </c>
       <c r="F53" t="n">
-        <v>-0.001539772654373816</v>
+        <v>0.009207904093122981</v>
       </c>
     </row>
     <row r="54">
@@ -2544,16 +2544,16 @@
         <v>-0.05550433232821735</v>
       </c>
       <c r="C54" t="n">
-        <v>-0.03803133153984457</v>
+        <v>-0.04163098759728212</v>
       </c>
       <c r="D54" t="n">
         <v>-0.04379614011242528</v>
       </c>
       <c r="E54" t="n">
-        <v>-0.04400992762642011</v>
+        <v>-0.05384011557774579</v>
       </c>
       <c r="F54" t="n">
-        <v>-0.04376008737320442</v>
+        <v>-0.05549477290482532</v>
       </c>
     </row>
     <row r="55">
@@ -2564,16 +2564,16 @@
         <v>-0.03441991477683013</v>
       </c>
       <c r="C55" t="n">
-        <v>-0.03452021977337541</v>
+        <v>-0.0350076919881742</v>
       </c>
       <c r="D55" t="n">
         <v>-0.03727713089984806</v>
       </c>
       <c r="E55" t="n">
-        <v>-0.03723453392861102</v>
+        <v>-0.08692177660110464</v>
       </c>
       <c r="F55" t="n">
-        <v>-0.03726049357484069</v>
+        <v>-0.08819313832499487</v>
       </c>
     </row>
     <row r="56">
@@ -2584,16 +2584,16 @@
         <v>0.01491953329812574</v>
       </c>
       <c r="C56" t="n">
-        <v>0.009656453254783955</v>
+        <v>0.01164498473639375</v>
       </c>
       <c r="D56" t="n">
         <v>0.03580369355824013</v>
       </c>
       <c r="E56" t="n">
-        <v>0.03549720191396255</v>
+        <v>0.04723789073710605</v>
       </c>
       <c r="F56" t="n">
-        <v>0.03469096010983312</v>
+        <v>0.04598464339974907</v>
       </c>
     </row>
     <row r="57">
@@ -2604,16 +2604,16 @@
         <v>-0.009778611968786882</v>
       </c>
       <c r="C57" t="n">
-        <v>0.003918579371541902</v>
+        <v>0.001646870630692012</v>
       </c>
       <c r="D57" t="n">
         <v>-0.01683805800516765</v>
       </c>
       <c r="E57" t="n">
-        <v>-0.01728369216645055</v>
+        <v>0.002997430667804013</v>
       </c>
       <c r="F57" t="n">
-        <v>-0.01838911741849573</v>
+        <v>0.003699386315050282</v>
       </c>
     </row>
     <row r="58">
@@ -2624,16 +2624,16 @@
         <v>0.009075954163016309</v>
       </c>
       <c r="C58" t="n">
-        <v>0.006521501823104808</v>
+        <v>0.007047251949108975</v>
       </c>
       <c r="D58" t="n">
         <v>0.01082714347627491</v>
       </c>
       <c r="E58" t="n">
-        <v>0.01152703736461851</v>
+        <v>-0.005144160208930815</v>
       </c>
       <c r="F58" t="n">
-        <v>0.01169005840875092</v>
+        <v>-0.008309911392587362</v>
       </c>
     </row>
     <row r="59">
@@ -2644,16 +2644,16 @@
         <v>-0.05253338545020794</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.04570494749237972</v>
+        <v>-0.04688492544302621</v>
       </c>
       <c r="D59" t="n">
         <v>-0.08162448270734325</v>
       </c>
       <c r="E59" t="n">
-        <v>-0.08100797566463623</v>
+        <v>-0.09338345805775487</v>
       </c>
       <c r="F59" t="n">
-        <v>-0.08069856914192382</v>
+        <v>-0.09472535994426688</v>
       </c>
     </row>
     <row r="60">
@@ -2664,16 +2664,16 @@
         <v>0.02153674073488552</v>
       </c>
       <c r="C60" t="n">
-        <v>0.01810933618382642</v>
+        <v>0.01959470068991066</v>
       </c>
       <c r="D60" t="n">
         <v>0.03803461615174045</v>
       </c>
       <c r="E60" t="n">
-        <v>0.03739854149356688</v>
+        <v>0.05504891334228443</v>
       </c>
       <c r="F60" t="n">
-        <v>0.03805179364162781</v>
+        <v>0.05720873662159766</v>
       </c>
     </row>
     <row r="61">
@@ -2684,16 +2684,16 @@
         <v>0.01953264768293812</v>
       </c>
       <c r="C61" t="n">
-        <v>0.0248423920228287</v>
+        <v>0.02386535050397324</v>
       </c>
       <c r="D61" t="n">
         <v>-0.01726815205799227</v>
       </c>
       <c r="E61" t="n">
-        <v>-0.01671386221670257</v>
+        <v>-0.007472064421585625</v>
       </c>
       <c r="F61" t="n">
-        <v>-0.0161627402056045</v>
+        <v>-0.006451987690851478</v>
       </c>
     </row>
     <row r="62">
@@ -2704,16 +2704,16 @@
         <v>0.03661054386609895</v>
       </c>
       <c r="C62" t="n">
-        <v>0.01535184619883256</v>
+        <v>0.01689962849383717</v>
       </c>
       <c r="D62" t="n">
         <v>0.07603690863090601</v>
       </c>
       <c r="E62" t="n">
-        <v>0.07655157454328584</v>
+        <v>0.0628645300526491</v>
       </c>
       <c r="F62" t="n">
-        <v>0.07717728933908784</v>
+        <v>0.06491203163483564</v>
       </c>
     </row>
     <row r="63">
@@ -2724,16 +2724,16 @@
         <v>0.02240286231202886</v>
       </c>
       <c r="C63" t="n">
-        <v>0.01923378636545168</v>
+        <v>0.02072040111880265</v>
       </c>
       <c r="D63" t="n">
         <v>-0.001483284179754729</v>
       </c>
       <c r="E63" t="n">
-        <v>-0.001298484164150258</v>
+        <v>0.01562495961399968</v>
       </c>
       <c r="F63" t="n">
-        <v>-0.001174661901892123</v>
+        <v>0.01415350918828506</v>
       </c>
     </row>
     <row r="64">
@@ -2744,16 +2744,16 @@
         <v>0.008917643301495151</v>
       </c>
       <c r="C64" t="n">
-        <v>0.01009566138397246</v>
+        <v>0.01004476219192293</v>
       </c>
       <c r="D64" t="n">
         <v>0.01296987343877379</v>
       </c>
       <c r="E64" t="n">
-        <v>0.01287540283032047</v>
+        <v>0.02999224187281031</v>
       </c>
       <c r="F64" t="n">
-        <v>0.01259863648591189</v>
+        <v>0.03314776679586603</v>
       </c>
     </row>
     <row r="65">
@@ -2764,16 +2764,16 @@
         <v>0.008073205459912745</v>
       </c>
       <c r="C65" t="n">
-        <v>0.006064988563398772</v>
+        <v>0.00451194108539171</v>
       </c>
       <c r="D65" t="n">
         <v>0.02224224988959288</v>
       </c>
       <c r="E65" t="n">
-        <v>0.022460160385442</v>
+        <v>-0.005781566785262777</v>
       </c>
       <c r="F65" t="n">
-        <v>0.02261462314819138</v>
+        <v>-0.005871047857828794</v>
       </c>
     </row>
     <row r="66">
@@ -2784,16 +2784,16 @@
         <v>-0.01124132435997483</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.01633043539403196</v>
+        <v>-0.01464144576679453</v>
       </c>
       <c r="D66" t="n">
         <v>-0.04731589556520111</v>
       </c>
       <c r="E66" t="n">
-        <v>-0.0466295995884843</v>
+        <v>-0.03973422349162674</v>
       </c>
       <c r="F66" t="n">
-        <v>-0.04670447372404288</v>
+        <v>-0.03874387993750737</v>
       </c>
     </row>
     <row r="67">
@@ -2804,16 +2804,16 @@
         <v>0.0437354968493094</v>
       </c>
       <c r="C67" t="n">
-        <v>0.0345734247329255</v>
+        <v>0.03484287173856972</v>
       </c>
       <c r="D67" t="n">
         <v>0.05641209010605747</v>
       </c>
       <c r="E67" t="n">
-        <v>0.05661230729568466</v>
+        <v>0.04403680791571642</v>
       </c>
       <c r="F67" t="n">
-        <v>0.05693526556377675</v>
+        <v>0.04158074888706375</v>
       </c>
     </row>
     <row r="68">
@@ -2824,16 +2824,16 @@
         <v>-0.005286450978308898</v>
       </c>
       <c r="C68" t="n">
-        <v>-0.01066378969046979</v>
+        <v>-0.00988516076536248</v>
       </c>
       <c r="D68" t="n">
         <v>-0.01440008118544814</v>
       </c>
       <c r="E68" t="n">
-        <v>-0.01440866017095315</v>
+        <v>-0.03684845249992264</v>
       </c>
       <c r="F68" t="n">
-        <v>-0.01414139299562778</v>
+        <v>-0.031101879800801</v>
       </c>
     </row>
     <row r="69">
@@ -2844,16 +2844,16 @@
         <v>0.01914790261286416</v>
       </c>
       <c r="C69" t="n">
-        <v>0.009676701392008135</v>
+        <v>0.01086956630630797</v>
       </c>
       <c r="D69" t="n">
         <v>-0.05710121097500874</v>
       </c>
       <c r="E69" t="n">
-        <v>-0.05701162919820932</v>
+        <v>-0.04245482597067289</v>
       </c>
       <c r="F69" t="n">
-        <v>-0.05708549680625066</v>
+        <v>-0.04394834244507345</v>
       </c>
     </row>
     <row r="70">
@@ -2864,16 +2864,16 @@
         <v>0.02627845191585233</v>
       </c>
       <c r="C70" t="n">
-        <v>0.03158412217726856</v>
+        <v>0.03336099881895378</v>
       </c>
       <c r="D70" t="n">
         <v>0.03038971883415154</v>
       </c>
       <c r="E70" t="n">
-        <v>0.03101060570992603</v>
+        <v>0.03215686757302565</v>
       </c>
       <c r="F70" t="n">
-        <v>0.03176897905099606</v>
+        <v>0.03047623156577581</v>
       </c>
     </row>
     <row r="71">
@@ -2884,16 +2884,16 @@
         <v>0.02962166351179261</v>
       </c>
       <c r="C71" t="n">
-        <v>0.02680399620275884</v>
+        <v>0.02524431562730694</v>
       </c>
       <c r="D71" t="n">
         <v>0.03558394552960962</v>
       </c>
       <c r="E71" t="n">
-        <v>0.03615359904266254</v>
+        <v>0.02388144148332137</v>
       </c>
       <c r="F71" t="n">
-        <v>0.03688440695339119</v>
+        <v>0.02594366786409288</v>
       </c>
     </row>
     <row r="72">
@@ -2904,16 +2904,16 @@
         <v>-0.03493622720370018</v>
       </c>
       <c r="C72" t="n">
-        <v>-0.02900481160745587</v>
+        <v>-0.02831267726221318</v>
       </c>
       <c r="D72" t="n">
         <v>-0.01065678404993961</v>
       </c>
       <c r="E72" t="n">
-        <v>-0.01082147892177804</v>
+        <v>-0.02216164429511746</v>
       </c>
       <c r="F72" t="n">
-        <v>-0.01080740076102908</v>
+        <v>-0.01847233643205141</v>
       </c>
     </row>
     <row r="73">
@@ -2924,16 +2924,16 @@
         <v>0.02927859986571662</v>
       </c>
       <c r="C73" t="n">
-        <v>0.02708874213826483</v>
+        <v>0.02769544771743743</v>
       </c>
       <c r="D73" t="n">
         <v>0.07206738650110425</v>
       </c>
       <c r="E73" t="n">
-        <v>0.07224731008700992</v>
+        <v>0.05386784751549158</v>
       </c>
       <c r="F73" t="n">
-        <v>0.07261995492904749</v>
+        <v>0.05360148774573594</v>
       </c>
     </row>
     <row r="74">
@@ -2944,16 +2944,16 @@
         <v>-0.0250283646518741</v>
       </c>
       <c r="C74" t="n">
-        <v>-0.01525733252196966</v>
+        <v>-0.014720293206404</v>
       </c>
       <c r="D74" t="n">
         <v>-0.0482064756652078</v>
       </c>
       <c r="E74" t="n">
-        <v>-0.04814171112320502</v>
+        <v>-0.05360502001279641</v>
       </c>
       <c r="F74" t="n">
-        <v>-0.0476415286027684</v>
+        <v>-0.05212953644418288</v>
       </c>
     </row>
     <row r="75">
@@ -2964,16 +2964,16 @@
         <v>-0.04248689147271349</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.03197424349919537</v>
+        <v>-0.03171670686100569</v>
       </c>
       <c r="D75" t="n">
         <v>-0.06670323746131065</v>
       </c>
       <c r="E75" t="n">
-        <v>-0.06644131358507933</v>
+        <v>-0.08229808365420146</v>
       </c>
       <c r="F75" t="n">
-        <v>-0.06555018649672266</v>
+        <v>-0.07882636473790945</v>
       </c>
     </row>
     <row r="76">
@@ -2984,16 +2984,16 @@
         <v>-0.05917456649142699</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.04738628101523908</v>
+        <v>-0.04928129296692574</v>
       </c>
       <c r="D76" t="n">
         <v>-0.1676063446518038</v>
       </c>
       <c r="E76" t="n">
-        <v>-0.1683417910390196</v>
+        <v>-0.1822807470465652</v>
       </c>
       <c r="F76" t="n">
-        <v>-0.1685355403138382</v>
+        <v>-0.1861834873545179</v>
       </c>
     </row>
     <row r="77">
@@ -3004,16 +3004,16 @@
         <v>0.1004174840674992</v>
       </c>
       <c r="C77" t="n">
-        <v>0.08632151713811889</v>
+        <v>0.08860672107207909</v>
       </c>
       <c r="D77" t="n">
         <v>0.09985373784843675</v>
       </c>
       <c r="E77" t="n">
-        <v>0.1001314795038582</v>
+        <v>0.1012296596674727</v>
       </c>
       <c r="F77" t="n">
-        <v>0.1003686257269625</v>
+        <v>0.1082315918423034</v>
       </c>
     </row>
     <row r="78">
@@ -3024,16 +3024,16 @@
         <v>0.007560993390064456</v>
       </c>
       <c r="C78" t="n">
-        <v>0.004427533037095157</v>
+        <v>0.0031205426230453</v>
       </c>
       <c r="D78" t="n">
         <v>0.004247792471245068</v>
       </c>
       <c r="E78" t="n">
-        <v>0.004030171059560441</v>
+        <v>0.01469524805442974</v>
       </c>
       <c r="F78" t="n">
-        <v>0.004183994749846667</v>
+        <v>0.009789759378085379</v>
       </c>
     </row>
     <row r="79">
@@ -3044,16 +3044,16 @@
         <v>0.06204307974958587</v>
       </c>
       <c r="C79" t="n">
-        <v>0.07357993260986952</v>
+        <v>0.07075572647440882</v>
       </c>
       <c r="D79" t="n">
         <v>0.06678052775027224</v>
       </c>
       <c r="E79" t="n">
-        <v>0.06727823087412949</v>
+        <v>0.05395234704807353</v>
       </c>
       <c r="F79" t="n">
-        <v>0.06922860636656544</v>
+        <v>0.0642518402203745</v>
       </c>
     </row>
     <row r="80">
@@ -3064,16 +3064,16 @@
         <v>0.03539191987199439</v>
       </c>
       <c r="C80" t="n">
-        <v>0.02660314230150895</v>
+        <v>0.02748009594305413</v>
       </c>
       <c r="D80" t="n">
         <v>0.07069760291997175</v>
       </c>
       <c r="E80" t="n">
-        <v>0.07063257740423498</v>
+        <v>0.05306175330401553</v>
       </c>
       <c r="F80" t="n">
-        <v>0.07119564366172854</v>
+        <v>0.0583091064213731</v>
       </c>
     </row>
     <row r="81">
@@ -3084,16 +3084,16 @@
         <v>-0.01487788946211403</v>
       </c>
       <c r="C81" t="n">
-        <v>-0.009356587717252462</v>
+        <v>-0.009334457254277487</v>
       </c>
       <c r="D81" t="n">
         <v>0.002963455062672685</v>
       </c>
       <c r="E81" t="n">
-        <v>0.002976201785582873</v>
+        <v>0.01343639088647794</v>
       </c>
       <c r="F81" t="n">
-        <v>0.002995320006721843</v>
+        <v>0.01189231116568985</v>
       </c>
     </row>
     <row r="82">
@@ -3104,16 +3104,16 @@
         <v>-0.0270982497928306</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.01821735781748086</v>
+        <v>-0.01901766759322636</v>
       </c>
       <c r="D82" t="n">
         <v>-0.01976019159151884</v>
       </c>
       <c r="E82" t="n">
-        <v>-0.01982734495013962</v>
+        <v>-0.009794560801310801</v>
       </c>
       <c r="F82" t="n">
-        <v>-0.01996090707452337</v>
+        <v>-0.01018507738244598</v>
       </c>
     </row>
     <row r="83">
@@ -3124,16 +3124,16 @@
         <v>0.02527055547972409</v>
       </c>
       <c r="C83" t="n">
-        <v>0.02911344488599499</v>
+        <v>0.03083523566080378</v>
       </c>
       <c r="D83" t="n">
         <v>0.02076694896278813</v>
       </c>
       <c r="E83" t="n">
-        <v>0.02054876991407237</v>
+        <v>0.0130946711800533</v>
       </c>
       <c r="F83" t="n">
-        <v>0.02142200123274267</v>
+        <v>0.0155430118474567</v>
       </c>
     </row>
     <row r="84">
@@ -3144,16 +3144,16 @@
         <v>0.04997765722030623</v>
       </c>
       <c r="C84" t="n">
-        <v>0.03337151018549741</v>
+        <v>0.03171402133412662</v>
       </c>
       <c r="D84" t="n">
         <v>0.1138726461826266</v>
       </c>
       <c r="E84" t="n">
-        <v>0.1145629405200037</v>
+        <v>0.1279201386457435</v>
       </c>
       <c r="F84" t="n">
-        <v>0.1143430579642278</v>
+        <v>0.1220971950661019</v>
       </c>
     </row>
     <row r="85">
@@ -3164,16 +3164,16 @@
         <v>0.02952371267760976</v>
       </c>
       <c r="C85" t="n">
-        <v>0.02768803892886611</v>
+        <v>0.02912515991638847</v>
       </c>
       <c r="D85" t="n">
         <v>0.0863300868375526</v>
       </c>
       <c r="E85" t="n">
-        <v>0.08644097003031621</v>
+        <v>0.07028940757266215</v>
       </c>
       <c r="F85" t="n">
-        <v>0.08633220822403539</v>
+        <v>0.07605027151833696</v>
       </c>
     </row>
     <row r="86">
@@ -3184,16 +3184,16 @@
         <v>-0.01240642626033056</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.003078812207042232</v>
+        <v>-0.008192719242621115</v>
       </c>
       <c r="D86" t="n">
         <v>0.0290323743679554</v>
       </c>
       <c r="E86" t="n">
-        <v>0.02929286548966377</v>
+        <v>0.006422595934550621</v>
       </c>
       <c r="F86" t="n">
-        <v>0.0298563700931061</v>
+        <v>0.006041512395913381</v>
       </c>
     </row>
     <row r="87">
@@ -3204,16 +3204,16 @@
         <v>0.01294189887641626</v>
       </c>
       <c r="C87" t="n">
-        <v>0.02037740568911604</v>
+        <v>0.01769735153787434</v>
       </c>
       <c r="D87" t="n">
         <v>0.0323510740028403</v>
       </c>
       <c r="E87" t="n">
-        <v>0.03198927303283507</v>
+        <v>0.0407187162120562</v>
       </c>
       <c r="F87" t="n">
-        <v>0.03093302694967932</v>
+        <v>0.03947275279871523</v>
       </c>
     </row>
     <row r="88">
@@ -3224,16 +3224,16 @@
         <v>0.03742807550493847</v>
       </c>
       <c r="C88" t="n">
-        <v>0.01700255004468775</v>
+        <v>0.01812558278090087</v>
       </c>
       <c r="D88" t="n">
         <v>0.001187989845889644</v>
       </c>
       <c r="E88" t="n">
-        <v>0.001168169126665411</v>
+        <v>-0.0157745189006309</v>
       </c>
       <c r="F88" t="n">
-        <v>0.0001770966026318254</v>
+        <v>-0.01410554445150366</v>
       </c>
     </row>
     <row r="89">
@@ -3244,16 +3244,16 @@
         <v>0.0005421055571272707</v>
       </c>
       <c r="C89" t="n">
-        <v>0.01526463789537858</v>
+        <v>0.01472057095990037</v>
       </c>
       <c r="D89" t="n">
         <v>0.0235277295748508</v>
       </c>
       <c r="E89" t="n">
-        <v>0.0237141006340784</v>
+        <v>0.03456136657664353</v>
       </c>
       <c r="F89" t="n">
-        <v>0.02356560022472544</v>
+        <v>0.03549720177797883</v>
       </c>
     </row>
     <row r="90">
@@ -3264,16 +3264,16 @@
         <v>0.007174088572342188</v>
       </c>
       <c r="C90" t="n">
-        <v>0.01177922088369703</v>
+        <v>0.009800158479754361</v>
       </c>
       <c r="D90" t="n">
         <v>0.03436338529690337</v>
       </c>
       <c r="E90" t="n">
-        <v>0.03436215063945153</v>
+        <v>0.02573266506218211</v>
       </c>
       <c r="F90" t="n">
-        <v>0.03395181164285317</v>
+        <v>0.02535310601339845</v>
       </c>
     </row>
     <row r="91">
@@ -3284,16 +3284,16 @@
         <v>0.006665569391887116</v>
       </c>
       <c r="C91" t="n">
-        <v>0.003150255345574803</v>
+        <v>0.007520733780095011</v>
       </c>
       <c r="D91" t="n">
         <v>-0.005238501108997855</v>
       </c>
       <c r="E91" t="n">
-        <v>-0.006168168979391209</v>
+        <v>0.01514982768052382</v>
       </c>
       <c r="F91" t="n">
-        <v>-0.007778469450801977</v>
+        <v>0.01473545415190072</v>
       </c>
     </row>
     <row r="92">
@@ -3304,16 +3304,16 @@
         <v>-0.001684561433368849</v>
       </c>
       <c r="C92" t="n">
-        <v>-0.005051305821833678</v>
+        <v>-0.002710987219425831</v>
       </c>
       <c r="D92" t="n">
         <v>-0.04397554540412282</v>
       </c>
       <c r="E92" t="n">
-        <v>-0.04405912543873529</v>
+        <v>-0.05053720637839446</v>
       </c>
       <c r="F92" t="n">
-        <v>-0.0440639964404784</v>
+        <v>-0.05048022887009829</v>
       </c>
     </row>
     <row r="93">
@@ -3324,16 +3324,16 @@
         <v>0.02320069799601338</v>
       </c>
       <c r="C93" t="n">
-        <v>0.01915520403412475</v>
+        <v>0.02601982158056717</v>
       </c>
       <c r="D93" t="n">
         <v>0.03903511321882387</v>
       </c>
       <c r="E93" t="n">
-        <v>0.038224931928058</v>
+        <v>0.08113794561458401</v>
       </c>
       <c r="F93" t="n">
-        <v>0.03780479428145199</v>
+        <v>0.08112681660805862</v>
       </c>
     </row>
     <row r="94">
@@ -3344,16 +3344,16 @@
         <v>-0.00813347172338306</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.009858877011871344</v>
+        <v>-0.009905662727891626</v>
       </c>
       <c r="D94" t="n">
         <v>-0.02352828398363307</v>
       </c>
       <c r="E94" t="n">
-        <v>-0.02390885362860802</v>
+        <v>-0.03272677760793286</v>
       </c>
       <c r="F94" t="n">
-        <v>-0.02429405549794846</v>
+        <v>-0.03404310986152283</v>
       </c>
     </row>
     <row r="95">
@@ -3364,16 +3364,16 @@
         <v>0.01753800021027732</v>
       </c>
       <c r="C95" t="n">
-        <v>0.01974566278437944</v>
+        <v>0.01958346264538322</v>
       </c>
       <c r="D95" t="n">
         <v>0.008119557267448457</v>
       </c>
       <c r="E95" t="n">
-        <v>0.00775755100607706</v>
+        <v>-0.01085124078532092</v>
       </c>
       <c r="F95" t="n">
-        <v>0.009391427606142302</v>
+        <v>-0.01067477463859935</v>
       </c>
     </row>
     <row r="96">
@@ -3384,16 +3384,16 @@
         <v>-0.006138495822780811</v>
       </c>
       <c r="C96" t="n">
-        <v>0.00276597530698398</v>
+        <v>0.001023787136840603</v>
       </c>
       <c r="D96" t="n">
         <v>-0.03487057144530385</v>
       </c>
       <c r="E96" t="n">
-        <v>-0.03524326178899736</v>
+        <v>0.02031623849834291</v>
       </c>
       <c r="F96" t="n">
-        <v>-0.03524505710721787</v>
+        <v>0.02011371611261755</v>
       </c>
     </row>
     <row r="97">
@@ -3404,16 +3404,16 @@
         <v>0.01908879116143317</v>
       </c>
       <c r="C97" t="n">
-        <v>0.01936120172823916</v>
+        <v>0.01818525724722557</v>
       </c>
       <c r="D97" t="n">
         <v>0.03877293711315413</v>
       </c>
       <c r="E97" t="n">
-        <v>0.03926005628528552</v>
+        <v>0.01352402698491554</v>
       </c>
       <c r="F97" t="n">
-        <v>0.03861203123566451</v>
+        <v>0.01450054531040299</v>
       </c>
     </row>
     <row r="98">
@@ -3424,16 +3424,16 @@
         <v>-0.0044162790328264</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.001726358705859183</v>
+        <v>-0.002836725520494457</v>
       </c>
       <c r="D98" t="n">
         <v>0.002924092229436752</v>
       </c>
       <c r="E98" t="n">
-        <v>-0.06818642534112243</v>
+        <v>-0.06734614725026108</v>
       </c>
       <c r="F98" t="n">
-        <v>-0.06806093030894465</v>
+        <v>-0.06785257737178109</v>
       </c>
     </row>
     <row r="99">
@@ -3444,16 +3444,16 @@
         <v>0.005929697681808897</v>
       </c>
       <c r="C99" t="n">
-        <v>0.0152026615836916</v>
+        <v>0.01216581570326179</v>
       </c>
       <c r="D99" t="n">
         <v>-0.04678409171731265</v>
       </c>
       <c r="E99" t="n">
-        <v>0.03641386019776357</v>
+        <v>0.03552412810645984</v>
       </c>
       <c r="F99" t="n">
-        <v>0.03664814472648414</v>
+        <v>0.03674392912298514</v>
       </c>
     </row>
     <row r="100">
@@ -3464,16 +3464,16 @@
         <v>0.002369401647356605</v>
       </c>
       <c r="C100" t="n">
-        <v>0.00125488764068313</v>
+        <v>0.00160764338755842</v>
       </c>
       <c r="D100" t="n">
         <v>0.02160171429843119</v>
       </c>
       <c r="E100" t="n">
-        <v>0.01316562175696337</v>
+        <v>0.01306456777389523</v>
       </c>
       <c r="F100" t="n">
-        <v>0.01327738970801542</v>
+        <v>0.01359740176955961</v>
       </c>
     </row>
     <row r="101">
@@ -3484,16 +3484,16 @@
         <v>-0.009432437794156326</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.01964601784570686</v>
+        <v>-0.0207357434841176</v>
       </c>
       <c r="D101" t="n">
         <v>-0.04929689726997008</v>
       </c>
       <c r="E101" t="n">
-        <v>-0.062842180935541</v>
+        <v>-0.06205579787862235</v>
       </c>
       <c r="F101" t="n">
-        <v>-0.06418264535546966</v>
+        <v>-0.06444050879086899</v>
       </c>
     </row>
     <row r="102">
@@ -3504,16 +3504,16 @@
         <v>-0.00326510997410868</v>
       </c>
       <c r="C102" t="n">
-        <v>-0.007728526215387227</v>
+        <v>-0.007160321798148543</v>
       </c>
       <c r="D102" t="n">
         <v>0.009638364803493562</v>
       </c>
       <c r="E102" t="n">
-        <v>0.0558396256053388</v>
+        <v>0.05568308749813149</v>
       </c>
       <c r="F102" t="n">
-        <v>0.05636940889517746</v>
+        <v>0.05650924025943835</v>
       </c>
     </row>
     <row r="103">
@@ -3524,16 +3524,16 @@
         <v>-0.03376211178309475</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.04193489740037034</v>
+        <v>-0.0429183154983077</v>
       </c>
       <c r="D103" t="n">
         <v>-0.07940058726618622</v>
       </c>
       <c r="E103" t="n">
-        <v>-0.1554972957886153</v>
+        <v>-0.1536460654876327</v>
       </c>
       <c r="F103" t="n">
-        <v>-0.1547733916231154</v>
+        <v>-0.1543775344572068</v>
       </c>
     </row>
     <row r="104">
@@ -3544,16 +3544,16 @@
         <v>0.007045676376755605</v>
       </c>
       <c r="C104" t="n">
-        <v>0.005796736973919493</v>
+        <v>0.007452075713098021</v>
       </c>
       <c r="D104" t="n">
         <v>0.00225283218921265</v>
       </c>
       <c r="E104" t="n">
-        <v>0.06958658037657681</v>
+        <v>0.07045716087701398</v>
       </c>
       <c r="F104" t="n">
-        <v>0.06994212451452014</v>
+        <v>0.06985669594438532</v>
       </c>
     </row>
     <row r="105">
@@ -3564,16 +3564,16 @@
         <v>-0.004344407317424614</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.008939190777243911</v>
+        <v>-0.008169509424144811</v>
       </c>
       <c r="D105" t="n">
         <v>0.0194592200082402</v>
       </c>
       <c r="E105" t="n">
-        <v>-0.01224388511476711</v>
+        <v>-0.01051733017082848</v>
       </c>
       <c r="F105" t="n">
-        <v>-0.01271262292825064</v>
+        <v>-0.01323493452651009</v>
       </c>
     </row>
     <row r="106">
@@ -3584,16 +3584,16 @@
         <v>-0.04716076525371982</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.06230844956205725</v>
+        <v>-0.05972265468381792</v>
       </c>
       <c r="D106" t="n">
         <v>-0.1019411321476542</v>
       </c>
       <c r="E106" t="n">
-        <v>-0.0663105559418883</v>
+        <v>-0.06334984458959762</v>
       </c>
       <c r="F106" t="n">
-        <v>-0.0650037682522293</v>
+        <v>-0.06355502095712652</v>
       </c>
     </row>
     <row r="107">
@@ -3604,16 +3604,16 @@
         <v>-0.02898275129818562</v>
       </c>
       <c r="C107" t="n">
-        <v>-0.02814948197415711</v>
+        <v>-0.02648858960876268</v>
       </c>
       <c r="D107" t="n">
         <v>0.001203819237218551</v>
       </c>
       <c r="E107" t="n">
-        <v>0.06346821651571173</v>
+        <v>0.06036266004725147</v>
       </c>
       <c r="F107" t="n">
-        <v>0.0627633863405155</v>
+        <v>0.06206601091296968</v>
       </c>
     </row>
     <row r="108">
@@ -3624,16 +3624,16 @@
         <v>0.1367273068063817</v>
       </c>
       <c r="C108" t="n">
-        <v>0.1342691177382868</v>
+        <v>0.1406317580718351</v>
       </c>
       <c r="D108" t="n">
         <v>0.13016429684924</v>
       </c>
       <c r="E108" t="n">
-        <v>0.1450830455831827</v>
+        <v>0.1428412278334507</v>
       </c>
       <c r="F108" t="n">
-        <v>0.143921863328095</v>
+        <v>0.1418298865892806</v>
       </c>
     </row>
     <row r="109">
@@ -3644,16 +3644,16 @@
         <v>-0.03505579172725707</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.02271319066397265</v>
+        <v>-0.02389441107283266</v>
       </c>
       <c r="D109" t="n">
         <v>-0.02161397376045171</v>
       </c>
       <c r="E109" t="n">
-        <v>-0.04764171068005165</v>
+        <v>-0.04502267332067049</v>
       </c>
       <c r="F109" t="n">
-        <v>-0.04845241825410039</v>
+        <v>-0.04694259910134576</v>
       </c>
     </row>
     <row r="110">
@@ -3664,16 +3664,16 @@
         <v>0.02969206256979659</v>
       </c>
       <c r="C110" t="n">
-        <v>0.02618283585428612</v>
+        <v>0.02838474945720569</v>
       </c>
       <c r="D110" t="n">
         <v>0.06590833620845173</v>
       </c>
       <c r="E110" t="n">
-        <v>0.04359349147056228</v>
+        <v>0.0399676044845206</v>
       </c>
       <c r="F110" t="n">
-        <v>0.044764355313916</v>
+        <v>0.04074385398135238</v>
       </c>
     </row>
     <row r="111">
@@ -3684,16 +3684,16 @@
         <v>-0.0003239717758208166</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.005257600241956875</v>
+        <v>-0.002352982935701436</v>
       </c>
       <c r="D111" t="n">
         <v>-0.04502747129102448</v>
       </c>
       <c r="E111" t="n">
-        <v>-0.001511536898894369</v>
+        <v>-0.004694319871754705</v>
       </c>
       <c r="F111" t="n">
-        <v>-0.001492687064264547</v>
+        <v>-0.005623153862255443</v>
       </c>
     </row>
     <row r="112">
@@ -3704,16 +3704,16 @@
         <v>0.03433484292635736</v>
       </c>
       <c r="C112" t="n">
-        <v>0.03681389118168362</v>
+        <v>0.0382946044285689</v>
       </c>
       <c r="D112" t="n">
         <v>0.03462702520974735</v>
       </c>
       <c r="E112" t="n">
-        <v>0.03771465824376787</v>
+        <v>0.03671393747296912</v>
       </c>
       <c r="F112" t="n">
-        <v>0.03766941833722231</v>
+        <v>0.03654644249552932</v>
       </c>
     </row>
     <row r="113">
@@ -3724,16 +3724,16 @@
         <v>0.0328453193394511</v>
       </c>
       <c r="C113" t="n">
-        <v>0.03409781193968847</v>
+        <v>0.03550802679482965</v>
       </c>
       <c r="D113" t="n">
         <v>0.006221408189294738</v>
       </c>
       <c r="E113" t="n">
-        <v>-0.02440439653963869</v>
+        <v>-0.02665034014876841</v>
       </c>
       <c r="F113" t="n">
-        <v>-0.02452865220240498</v>
+        <v>-0.0267576999163679</v>
       </c>
     </row>
     <row r="114">
@@ -3744,16 +3744,16 @@
         <v>0.02117642596643819</v>
       </c>
       <c r="C114" t="n">
-        <v>0.01207039089213772</v>
+        <v>0.02191706863305706</v>
       </c>
       <c r="D114" t="n">
         <v>-0.001498942229409791</v>
       </c>
       <c r="E114" t="n">
-        <v>0.04374173228056276</v>
+        <v>0.04423673504761276</v>
       </c>
       <c r="F114" t="n">
-        <v>0.04319605589241214</v>
+        <v>0.04403103666780343</v>
       </c>
     </row>
     <row r="115">
@@ -3764,16 +3764,16 @@
         <v>0.002255221227168348</v>
       </c>
       <c r="C115" t="n">
-        <v>-0.01154604883911889</v>
+        <v>-0.007602341041122713</v>
       </c>
       <c r="D115" t="n">
         <v>0.03338471222996842</v>
       </c>
       <c r="E115" t="n">
-        <v>0.03497633061734438</v>
+        <v>0.03569452538904459</v>
       </c>
       <c r="F115" t="n">
-        <v>0.03449403625621112</v>
+        <v>0.03519828463388248</v>
       </c>
     </row>
     <row r="116">
@@ -3784,16 +3784,16 @@
         <v>0.02470330263373569</v>
       </c>
       <c r="C116" t="n">
-        <v>0.02037267079270273</v>
+        <v>0.01341795458808248</v>
       </c>
       <c r="D116" t="n">
         <v>0.0403096139031283</v>
       </c>
       <c r="E116" t="n">
-        <v>0.03010155399498732</v>
+        <v>0.03271934823092206</v>
       </c>
       <c r="F116" t="n">
-        <v>0.02948779060805379</v>
+        <v>0.03231390769152861</v>
       </c>
     </row>
     <row r="117">
@@ -3804,16 +3804,16 @@
         <v>-0.03108599772549688</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.02459471821514291</v>
+        <v>-0.02844239397135058</v>
       </c>
       <c r="D117" t="n">
         <v>-0.04637740616986598</v>
       </c>
       <c r="E117" t="n">
-        <v>-0.00794534065213532</v>
+        <v>-0.01156231657158641</v>
       </c>
       <c r="F117" t="n">
-        <v>-0.008764724849543895</v>
+        <v>-0.01291110771460489</v>
       </c>
     </row>
     <row r="118">
@@ -3824,16 +3824,16 @@
         <v>-0.0194945890245552</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.02083460188856142</v>
+        <v>-0.02194033719833173</v>
       </c>
       <c r="D118" t="n">
         <v>-0.0131917396815385</v>
       </c>
       <c r="E118" t="n">
-        <v>-0.02651552404033563</v>
+        <v>-0.02921400217322997</v>
       </c>
       <c r="F118" t="n">
-        <v>-0.02667011230061712</v>
+        <v>-0.02929835980836795</v>
       </c>
     </row>
     <row r="119">
@@ -3844,16 +3844,16 @@
         <v>-0.022664548253229</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.01996249287119488</v>
+        <v>-0.01770893269221524</v>
       </c>
       <c r="D119" t="n">
         <v>-0.03193660996460233</v>
       </c>
       <c r="E119" t="n">
-        <v>-0.004433265236199197</v>
+        <v>-0.007339529168892405</v>
       </c>
       <c r="F119" t="n">
-        <v>-0.004545243191141741</v>
+        <v>-0.007856584974253634</v>
       </c>
     </row>
     <row r="120">
@@ -3864,16 +3864,16 @@
         <v>0.06364275547966883</v>
       </c>
       <c r="C120" t="n">
-        <v>0.06272213259369087</v>
+        <v>0.06879270521953884</v>
       </c>
       <c r="D120" t="n">
         <v>0.07971419850955186</v>
       </c>
       <c r="E120" t="n">
-        <v>0.1033283801639431</v>
+        <v>0.1033756493991741</v>
       </c>
       <c r="F120" t="n">
-        <v>0.1017737650780341</v>
+        <v>0.1015840256684916</v>
       </c>
     </row>
     <row r="121">
@@ -3884,16 +3884,16 @@
         <v>0.03759026104415096</v>
       </c>
       <c r="C121" t="n">
-        <v>0.03189980455009726</v>
+        <v>0.03038411715589851</v>
       </c>
       <c r="D121" t="n">
         <v>0.04703396367444367</v>
       </c>
       <c r="E121" t="n">
-        <v>0.05992508829756442</v>
+        <v>0.05838950102409952</v>
       </c>
       <c r="F121" t="n">
-        <v>0.05614505207078475</v>
+        <v>0.05378134391112208</v>
       </c>
     </row>
     <row r="122">
@@ -3904,16 +3904,16 @@
         <v>-0.007217413861557577</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.003607274038559656</v>
+        <v>-0.003768452014982</v>
       </c>
       <c r="D122" t="n">
         <v>-0.01585787527416958</v>
       </c>
       <c r="E122" t="n">
-        <v>-0.01436713067645246</v>
+        <v>-0.01446796969677161</v>
       </c>
       <c r="F122" t="n">
-        <v>-0.01581384260967626</v>
+        <v>-0.01578960343330149</v>
       </c>
     </row>
     <row r="123">
@@ -3924,16 +3924,16 @@
         <v>-0.004342256575710102</v>
       </c>
       <c r="C123" t="n">
-        <v>-0.00507304469177586</v>
+        <v>-0.00623701494340292</v>
       </c>
       <c r="D123" t="n">
         <v>0.03022495642883836</v>
       </c>
       <c r="E123" t="n">
-        <v>0.07773376899709671</v>
+        <v>0.07777095681460536</v>
       </c>
       <c r="F123" t="n">
-        <v>0.07773738828323981</v>
+        <v>0.07775722888334399</v>
       </c>
     </row>
     <row r="124">
@@ -3944,16 +3944,16 @@
         <v>-0.01953843393865837</v>
       </c>
       <c r="C124" t="n">
-        <v>-0.02776727215230595</v>
+        <v>-0.02858311747226601</v>
       </c>
       <c r="D124" t="n">
         <v>0.02917740961821971</v>
       </c>
       <c r="E124" t="n">
-        <v>0.02729568666036274</v>
+        <v>0.02723725776293216</v>
       </c>
       <c r="F124" t="n">
-        <v>0.02872523936374066</v>
+        <v>0.02878715510735425</v>
       </c>
     </row>
     <row r="125">
@@ -3964,16 +3964,16 @@
         <v>0.0161922377797206</v>
       </c>
       <c r="C125" t="n">
-        <v>-0.001033803811487254</v>
+        <v>0.001850403871937712</v>
       </c>
       <c r="D125" t="n">
         <v>0.01123730081200413</v>
       </c>
       <c r="E125" t="n">
-        <v>0.02264959298810279</v>
+        <v>0.02258581082007466</v>
       </c>
       <c r="F125" t="n">
-        <v>0.02199408796162773</v>
+        <v>0.02205122779016681</v>
       </c>
     </row>
     <row r="126">
@@ -3984,16 +3984,16 @@
         <v>0.008240643323985029</v>
       </c>
       <c r="C126" t="n">
-        <v>0.01492853645995951</v>
+        <v>0.01178722103447978</v>
       </c>
       <c r="D126" t="n">
         <v>0.01648872644524583</v>
       </c>
       <c r="E126" t="n">
-        <v>0.06254640071203323</v>
+        <v>0.06258050897089301</v>
       </c>
       <c r="F126" t="n">
-        <v>0.06530199892494754</v>
+        <v>0.06529818952948377</v>
       </c>
     </row>
     <row r="127">
@@ -4004,16 +4004,16 @@
         <v>-0.01724511257095454</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.02071061847046735</v>
+        <v>-0.01385681863938492</v>
       </c>
       <c r="D127" t="n">
         <v>0.0007354646659207265</v>
       </c>
       <c r="E127" t="n">
-        <v>0.008869713150363917</v>
+        <v>0.009215216573043482</v>
       </c>
       <c r="F127" t="n">
-        <v>0.01120005041983711</v>
+        <v>0.01115827279165665</v>
       </c>
     </row>
     <row r="128">
@@ -4024,16 +4024,16 @@
         <v>0.02113785160145753</v>
       </c>
       <c r="C128" t="n">
-        <v>0.01476590606249503</v>
+        <v>0.01830451561409212</v>
       </c>
       <c r="D128" t="n">
         <v>0.003334579349555053</v>
       </c>
       <c r="E128" t="n">
-        <v>0.1157998499760755</v>
+        <v>0.1158939966881361</v>
       </c>
       <c r="F128" t="n">
-        <v>0.1122386282875092</v>
+        <v>0.1119736120121387</v>
       </c>
     </row>
     <row r="129">
@@ -4044,16 +4044,16 @@
         <v>0.035985617226017</v>
       </c>
       <c r="C129" t="n">
-        <v>0.03747209078262993</v>
+        <v>0.04198317070116487</v>
       </c>
       <c r="D129" t="n">
         <v>0.01638387548657119</v>
       </c>
       <c r="E129" t="n">
-        <v>-0.003983278805989114</v>
+        <v>-0.00403554752050159</v>
       </c>
       <c r="F129" t="n">
-        <v>0.001912739149313137</v>
+        <v>0.001965191185640021</v>
       </c>
     </row>
     <row r="130">
@@ -4064,16 +4064,16 @@
         <v>0.05509212824741899</v>
       </c>
       <c r="C130" t="n">
-        <v>0.04700545301259507</v>
+        <v>0.0445844228500575</v>
       </c>
       <c r="D130" t="n">
         <v>0.033666084053502</v>
       </c>
       <c r="E130" t="n">
-        <v>-0.009691568712586487</v>
+        <v>-0.00980037773442749</v>
       </c>
       <c r="F130" t="n">
-        <v>-0.009187404449423082</v>
+        <v>-0.009035002239946757</v>
       </c>
     </row>
     <row r="131">
@@ -4084,16 +4084,16 @@
         <v>-0.008899448039595201</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.02991858995905984</v>
+        <v>-0.02743259343601396</v>
       </c>
       <c r="D131" t="n">
         <v>-0.04458566957284057</v>
       </c>
       <c r="E131" t="n">
-        <v>-0.02214683381130231</v>
+        <v>-0.02216195934066085</v>
       </c>
       <c r="F131" t="n">
-        <v>-0.02308278827818254</v>
+        <v>-0.0231011647070588</v>
       </c>
     </row>
     <row r="132">
@@ -4104,16 +4104,16 @@
         <v>-0.03019807292186837</v>
       </c>
       <c r="C132" t="n">
-        <v>-0.03855199494413762</v>
+        <v>-0.04058049761111916</v>
       </c>
       <c r="D132" t="n">
         <v>-0.02738335071421504</v>
       </c>
       <c r="E132" t="n">
-        <v>0.01300310584170821</v>
+        <v>0.01294234340921937</v>
       </c>
       <c r="F132" t="n">
-        <v>0.01080487680373115</v>
+        <v>0.01079557741776682</v>
       </c>
     </row>
     <row r="133">
@@ -4124,16 +4124,16 @@
         <v>0.004458709194749865</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.004590812401806413</v>
+        <v>-0.006059282173186955</v>
       </c>
       <c r="D133" t="n">
         <v>-0.003693654035491267</v>
       </c>
       <c r="E133" t="n">
-        <v>-0.1264263415735598</v>
+        <v>-0.1264954092637685</v>
       </c>
       <c r="F133" t="n">
-        <v>-0.1211944008906954</v>
+        <v>-0.1209099294972955</v>
       </c>
     </row>
     <row r="134">
@@ -4144,16 +4144,16 @@
         <v>-0.01012098237064429</v>
       </c>
       <c r="C134" t="n">
-        <v>-0.005195219651400633</v>
+        <v>-0.007177090906426156</v>
       </c>
       <c r="D134" t="n">
         <v>0.005809586069590342</v>
       </c>
       <c r="E134" t="n">
-        <v>0.005997168479109237</v>
+        <v>0.04679505621658709</v>
       </c>
       <c r="F134" t="n">
-        <v>0.01103066823236194</v>
+        <v>0.04921537197797584</v>
       </c>
     </row>
     <row r="135">
@@ -4164,16 +4164,16 @@
         <v>0.001975471124104984</v>
       </c>
       <c r="C135" t="n">
-        <v>0.01268933937821866</v>
+        <v>0.01218731926401682</v>
       </c>
       <c r="D135" t="n">
         <v>-0.01602392225709455</v>
       </c>
       <c r="E135" t="n">
-        <v>-0.01587368874369649</v>
+        <v>-0.05041275457708798</v>
       </c>
       <c r="F135" t="n">
-        <v>0.01511116995982982</v>
+        <v>-0.0509568772564145</v>
       </c>
     </row>
     <row r="136">
@@ -4184,16 +4184,16 @@
         <v>0.01197982270640709</v>
       </c>
       <c r="C136" t="n">
-        <v>0.001263495400050225</v>
+        <v>0.001818217553623354</v>
       </c>
       <c r="D136" t="n">
         <v>0.02116303136744554</v>
       </c>
       <c r="E136" t="n">
-        <v>0.02089816581657745</v>
+        <v>-0.03235743542231086</v>
       </c>
       <c r="F136" t="n">
-        <v>0.02520281734160204</v>
+        <v>-0.03109433081975167</v>
       </c>
     </row>
     <row r="137">
@@ -4204,16 +4204,16 @@
         <v>0.01107818091885257</v>
       </c>
       <c r="C137" t="n">
-        <v>0.01680571228875365</v>
+        <v>0.0161424315999742</v>
       </c>
       <c r="D137" t="n">
         <v>0.01716310963292009</v>
       </c>
       <c r="E137" t="n">
-        <v>0.01756427387733167</v>
+        <v>0.0501497402082383</v>
       </c>
       <c r="F137" t="n">
-        <v>-0.02297172906158039</v>
+        <v>0.05355534030325342</v>
       </c>
     </row>
     <row r="138">
@@ -4224,16 +4224,16 @@
         <v>0.0408748768225022</v>
       </c>
       <c r="C138" t="n">
-        <v>0.04410636877303806</v>
+        <v>0.04591922130687566</v>
       </c>
       <c r="D138" t="n">
         <v>0.04571108411379798</v>
       </c>
       <c r="E138" t="n">
-        <v>0.04553966677561974</v>
+        <v>0.05880163415834079</v>
       </c>
       <c r="F138" t="n">
-        <v>0.0344891447317336</v>
+        <v>0.06468864609971578</v>
       </c>
     </row>
     <row r="139">
@@ -4244,16 +4244,16 @@
         <v>0.02695355150691722</v>
       </c>
       <c r="C139" t="n">
-        <v>0.03461292617718791</v>
+        <v>0.03339890038979117</v>
       </c>
       <c r="D139" t="n">
         <v>0.05114499695263859</v>
       </c>
       <c r="E139" t="n">
-        <v>0.0525144181607627</v>
+        <v>0.06066987718095579</v>
       </c>
       <c r="F139" t="n">
-        <v>0.02348460396222714</v>
+        <v>0.06360214199853206</v>
       </c>
     </row>
     <row r="140">
@@ -4264,16 +4264,16 @@
         <v>0.001105337613598443</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.008273246827220779</v>
+        <v>-0.009182420491382922</v>
       </c>
       <c r="D140" t="n">
         <v>0.01207650834328272</v>
       </c>
       <c r="E140" t="n">
-        <v>0.01161572502720785</v>
+        <v>0.02715505333991364</v>
       </c>
       <c r="F140" t="n">
-        <v>0.0585585260358842</v>
+        <v>0.02688883590664632</v>
       </c>
     </row>
     <row r="141">
@@ -4284,16 +4284,16 @@
         <v>0.01548353080167544</v>
       </c>
       <c r="C141" t="n">
-        <v>0.01690332126514456</v>
+        <v>0.0166183869287236</v>
       </c>
       <c r="D141" t="n">
         <v>0.009490382556151769</v>
       </c>
       <c r="E141" t="n">
-        <v>0.009101264758885525</v>
+        <v>0.002284052534513192</v>
       </c>
       <c r="F141" t="n">
-        <v>0.0710984118561566</v>
+        <v>0.0009385649053456034</v>
       </c>
     </row>
     <row r="142">
@@ -4304,16 +4304,16 @@
         <v>0.02771801345839262</v>
       </c>
       <c r="C142" t="n">
-        <v>0.02501226988870403</v>
+        <v>0.0249215611614801</v>
       </c>
       <c r="D142" t="n">
         <v>0.05080959391353825</v>
       </c>
       <c r="E142" t="n">
-        <v>0.05086822561248006</v>
+        <v>0.04081114281988377</v>
       </c>
       <c r="F142" t="n">
-        <v>0.03312017975160703</v>
+        <v>0.04506476884369998</v>
       </c>
     </row>
     <row r="143">
@@ -4324,16 +4324,16 @@
         <v>0.03072733112833025</v>
       </c>
       <c r="C143" t="n">
-        <v>0.01696602722211408</v>
+        <v>0.01657810686811452</v>
       </c>
       <c r="D143" t="n">
         <v>0.0494642092634302</v>
       </c>
       <c r="E143" t="n">
-        <v>0.04945569757283717</v>
+        <v>0.1140986298914752</v>
       </c>
       <c r="F143" t="n">
-        <v>0.08989000870391231</v>
+        <v>0.1083709685256331</v>
       </c>
     </row>
     <row r="144">
@@ -4344,16 +4344,16 @@
         <v>0.005776013045626965</v>
       </c>
       <c r="C144" t="n">
-        <v>-0.0023032155579752</v>
+        <v>-0.001572638897650625</v>
       </c>
       <c r="D144" t="n">
         <v>-0.009290385971130546</v>
       </c>
       <c r="E144" t="n">
-        <v>-0.008711382628370679</v>
+        <v>-0.02094880186378198</v>
       </c>
       <c r="F144" t="n">
-        <v>-0.02104715530531</v>
+        <v>-0.02014346749149528</v>
       </c>
     </row>
     <row r="145">
@@ -4364,16 +4364,16 @@
         <v>0.01025740003853813</v>
       </c>
       <c r="C145" t="n">
-        <v>0.004676867327492213</v>
+        <v>0.007735709568713065</v>
       </c>
       <c r="D145" t="n">
         <v>0.03121426216286869</v>
       </c>
       <c r="E145" t="n">
-        <v>0.03129970256994376</v>
+        <v>0.02839343409114205</v>
       </c>
       <c r="F145" t="n">
-        <v>0.04208094155713056</v>
+        <v>0.02742781550990563</v>
       </c>
     </row>
   </sheetData>

</xml_diff>